<commit_message>
Adopt approved 47-hour Ephrata allocation and preserve observation gates
</commit_message>
<xml_diff>
--- a/ten_day_operating_plan.xlsx
+++ b/ten_day_operating_plan.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="1" r:id="R991860cc761644ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily plan" sheetId="2" r:id="R521d6b30e30440dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work log" sheetId="3" r:id="Reea858493b864dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="4" r:id="R11c25403661e4510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="1" r:id="R0a21d24682464ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily plan" sheetId="2" r:id="R989a0306a8794ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work log" sheetId="3" r:id="R32ec74fa6ea54fad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="4" r:id="R03a62d211d7546dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -529,7 +529,7 @@
       </x:c>
       <x:c r="C7" s="8" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$D$6:$D$74,A7,'Work log'!$E$6:$E$74,"&lt;&gt;Coverage")</x:f>
-        <x:v>31</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D7" s="8" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$D$6:$D$74,A7,'Work log'!$E$6:$E$74,"Coverage")</x:f>
@@ -537,11 +537,11 @@
       </x:c>
       <x:c r="E7" s="8" t="n">
         <x:f>SUM(C7:D7)</x:f>
-        <x:v>31</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F7" s="8" t="n">
         <x:f>B7-E7</x:f>
-        <x:v>5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G7" s="2" t="str">
         <x:f>IF(COUNTBLANK('Inputs'!B7)&gt;0,"MISSING INPUT",IF(B7&lt;0,"INVALID INPUT",IF(F7&lt;0,"OVER CAPACITY","OK")))</x:f>
@@ -645,7 +645,7 @@
       </x:c>
       <x:c r="C11" s="26" t="n">
         <x:f>SUM(C6:C10)</x:f>
-        <x:v>75.5</x:v>
+        <x:v>67.5</x:v>
       </x:c>
       <x:c r="D11" s="26" t="n">
         <x:f>SUM(D6:D10)</x:f>
@@ -653,11 +653,11 @@
       </x:c>
       <x:c r="E11" s="26" t="n">
         <x:f>SUM(E6:E10)</x:f>
-        <x:v>89.5</x:v>
+        <x:v>81.5</x:v>
       </x:c>
       <x:c r="F11" s="26" t="n">
         <x:f>SUM(F6:F10)</x:f>
-        <x:v>37</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G11" s="13"/>
     </x:row>
@@ -992,7 +992,7 @@
       </x:c>
       <x:c r="B33" s="8" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$E$6:$E$74,A33)</x:f>
-        <x:v>55</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C33" s="2"/>
       <x:c r="D33" s="2"/>
@@ -1081,7 +1081,7 @@
       </x:c>
       <x:c r="B39" s="8" t="n">
         <x:f>SUM(F6:F9)</x:f>
-        <x:v>22</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C39" s="2"/>
       <x:c r="D39" s="2"/>
@@ -2184,11 +2184,11 @@
       </x:c>
       <x:c r="F31" s="8" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$D$6:$D$74,C31,'Work log'!$B$6:$B$74,A31,'Work log'!$E$6:$E$74,"&lt;&gt;Coverage")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G31" s="8" t="n">
         <x:f>IF(ISNUMBER(E31),E31-F31,"")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H31" s="2" t="str">
         <x:f>IF(NOT(ISNUMBER(E31)),"MISSING",IF(E31&lt;0,"INVALID",IF(OR(B31&lt;'Inputs'!$B$14,B31&gt;'Inputs'!$B$15,WEEKDAY(B31,2)&gt;5,B31&lt;&gt;WORKDAY('Inputs'!$B$14,A31-1)),"DATE",IF(G31&lt;0,"OVER","OK"))))</x:f>
@@ -2388,11 +2388,11 @@
       </x:c>
       <x:c r="F37" s="24" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$D$6:$D$74,C37,'Work log'!$B$6:$B$74,A37,'Work log'!$E$6:$E$74,"&lt;&gt;Coverage")</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G37" s="24" t="n">
         <x:f>IF(ISNUMBER(E37),E37-F37,"")</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H37" s="20" t="str">
         <x:f>IF(NOT(ISNUMBER(E37)),"MISSING",IF(E37&lt;0,"INVALID",IF(OR(B37&lt;'Inputs'!$B$14,B37&gt;'Inputs'!$B$15,WEEKDAY(B37,2)&gt;5,B37&lt;&gt;WORKDAY('Inputs'!$B$14,A37-1)),"DATE",IF(G37&lt;0,"OVER","OK"))))</x:f>
@@ -2592,11 +2592,11 @@
       </x:c>
       <x:c r="F43" s="8" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$D$6:$D$74,C43,'Work log'!$B$6:$B$74,A43,'Work log'!$E$6:$E$74,"&lt;&gt;Coverage")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G43" s="8" t="n">
         <x:f>IF(ISNUMBER(E43),E43-F43,"")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H43" s="2" t="str">
         <x:f>IF(NOT(ISNUMBER(E43)),"MISSING",IF(E43&lt;0,"INVALID",IF(OR(B43&lt;'Inputs'!$B$14,B43&gt;'Inputs'!$B$15,WEEKDAY(B43,2)&gt;5,B43&lt;&gt;WORKDAY('Inputs'!$B$14,A43-1)),"DATE",IF(G43&lt;0,"OVER","OK"))))</x:f>
@@ -2796,11 +2796,11 @@
       </x:c>
       <x:c r="F49" s="24" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$D$6:$D$74,C49,'Work log'!$B$6:$B$74,A49,'Work log'!$E$6:$E$74,"&lt;&gt;Coverage")</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G49" s="24" t="n">
         <x:f>IF(ISNUMBER(E49),E49-F49,"")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H49" s="20" t="str">
         <x:f>IF(NOT(ISNUMBER(E49)),"MISSING",IF(E49&lt;0,"INVALID",IF(OR(B49&lt;'Inputs'!$B$14,B49&gt;'Inputs'!$B$15,WEEKDAY(B49,2)&gt;5,B49&lt;&gt;WORKDAY('Inputs'!$B$14,A49-1)),"DATE",IF(G49&lt;0,"OVER","OK"))))</x:f>
@@ -3000,11 +3000,11 @@
       </x:c>
       <x:c r="F55" s="8" t="n">
         <x:f>SUMIFS('Work log'!$F$6:$F$74,'Work log'!$D$6:$D$74,C55,'Work log'!$B$6:$B$74,A55,'Work log'!$E$6:$E$74,"&lt;&gt;Coverage")</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G55" s="8" t="n">
         <x:f>IF(ISNUMBER(E55),E55-F55,"")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H55" s="2" t="str">
         <x:f>IF(NOT(ISNUMBER(E55)),"MISSING",IF(E55&lt;0,"INVALID",IF(OR(B55&lt;'Inputs'!$B$14,B55&gt;'Inputs'!$B$15,WEEKDAY(B55,2)&gt;5,B55&lt;&gt;WORKDAY('Inputs'!$B$14,A55-1)),"DATE",IF(G55&lt;0,"OVER","OK"))))</x:f>
@@ -4908,7 +4908,7 @@
         <x:v>Ephrata</x:v>
       </x:c>
       <x:c r="F42" s="16" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G42" s="18" t="str">
         <x:v>Review weekend logs and morning sample 1</x:v>
@@ -5103,7 +5103,7 @@
         <x:v>Ephrata</x:v>
       </x:c>
       <x:c r="F47" s="16" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="18" t="str">
         <x:v>Review morning sample 2 and adoption exceptions</x:v>
@@ -5298,7 +5298,7 @@
         <x:v>Ephrata</x:v>
       </x:c>
       <x:c r="F52" s="16" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G52" s="18" t="str">
         <x:v>Review morning sample 3 and exceptions</x:v>
@@ -5532,7 +5532,7 @@
         <x:v>Ephrata</x:v>
       </x:c>
       <x:c r="F58" s="16" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G58" s="18" t="str">
         <x:v>Review sample 4 and rotation exposure</x:v>
@@ -5727,7 +5727,7 @@
         <x:v>Ephrata</x:v>
       </x:c>
       <x:c r="F63" s="16" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G63" s="18" t="str">
         <x:v>Review sample 5 and prepare acceptance packet</x:v>

</xml_diff>

<commit_message>
Require authorized Durant cutoff before final-day deactivation
</commit_message>
<xml_diff>
--- a/ten_day_operating_plan.xlsx
+++ b/ten_day_operating_plan.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="1" r:id="R0a21d24682464ad2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily plan" sheetId="2" r:id="R989a0306a8794ee1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work log" sheetId="3" r:id="R32ec74fa6ea54fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="4" r:id="R03a62d211d7546dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="1" r:id="R7b8f80faa2fb4447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily plan" sheetId="2" r:id="Rb95057e2f2fc4d54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work log" sheetId="3" r:id="R312783d4d0494c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="4" r:id="R79f0674eedef45fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5850,10 +5850,10 @@
         <x:v>Deactivate WellSky/Riley/Casey on agreed final day</x:v>
       </x:c>
       <x:c r="H66" s="18" t="str">
-        <x:v>Export handoff; approved documented checklist</x:v>
+        <x:v>Export handoff; approved checklist; authorized Sep 18 cutoff confirmed</x:v>
       </x:c>
       <x:c r="I66" s="18" t="str">
-        <x:v>Disconnected / disabled evidence</x:v>
+        <x:v>Disabled evidence at authorized cutoff; no early service end</x:v>
       </x:c>
       <x:c r="J66" s="19" t="str">
         <x:v>Planned</x:v>

</xml_diff>